<commit_message>
Update Excel dan index.html dengan data terbaru
</commit_message>
<xml_diff>
--- a/REKAP NILAIAN ASTS - Personal Branding XI DKV 2026-2027.xlsx
+++ b/REKAP NILAIAN ASTS - Personal Branding XI DKV 2026-2027.xlsx
@@ -1,105 +1,105 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="1. REKAP NILAI" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2. NILAI KOMPONEN" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Detail - Wahdan Sapari" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Detail - Ahmad Fauzi" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Detail - Qiandra Kaizar Nahari" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Detail - Ilma Latifah" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Detail - Sopa Anidatul Aisah" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Detail - Jajang M Husni Mubarok" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Detail - Silvi Budia Putri" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Detail - Nurjihan" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Detail - Dede Aprilia Kartika" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Detail - Putri Intan Nuraeni" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Detail - Intan Widiyanti" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Detail - Safinah Syara Garini" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Detail - Quinsya Rahmanesa Sole" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Detail - Jihan Shafira Kean Put" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Detail - Dhea Eka Khoerunnisa" sheetId="17" state="visible" r:id="rId17"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Detail - Wulan Sundari" sheetId="18" state="visible" r:id="rId18"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Detail - Wilda Azkia" sheetId="19" state="visible" r:id="rId19"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Detail - Muhamad Diaz Pirdaus" sheetId="20" state="visible" r:id="rId20"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Detail - Rizky Muhammad Regal S" sheetId="21" state="visible" r:id="rId21"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Detail - Khanza Nuraeni" sheetId="22" state="visible" r:id="rId22"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Detail - Ceisha Sinthia" sheetId="23" state="visible" r:id="rId23"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Detail - Selvi Sifa Urizqi" sheetId="24" state="visible" r:id="rId24"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Detail - Azmi Anugrah" sheetId="25" state="visible" r:id="rId25"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Detail - Indri Fitriyani" sheetId="26" state="visible" r:id="rId26"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Detail - Meisya Fakhriyah" sheetId="27" state="visible" r:id="rId27"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Detail - M Reza Huafah" sheetId="28" state="visible" r:id="rId28"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Detail - Syiva Widiyana Agustin" sheetId="29" state="visible" r:id="rId29"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Detail - Meylan Meliyanti Anast" sheetId="30" state="visible" r:id="rId30"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Detail - Putri Utami" sheetId="31" state="visible" r:id="rId31"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Detail - Kamila Apriliani" sheetId="32" state="visible" r:id="rId32"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Detail - Yayu Astia" sheetId="33" state="visible" r:id="rId33"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Detail - Wina Afriliani" sheetId="34" state="visible" r:id="rId34"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Detail - Jajang Nurjaman" sheetId="35" state="visible" r:id="rId35"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Detail - Shandika Revi Shafarud" sheetId="36" state="visible" r:id="rId36"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Detail - Ai Tito" sheetId="37" state="visible" r:id="rId37"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Detail - Merlin Aznika" sheetId="38" state="visible" r:id="rId38"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Detail - Neng Sri Rahayu" sheetId="39" state="visible" r:id="rId39"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Detail - Sindia Saputri" sheetId="40" state="visible" r:id="rId40"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Detail - Mutia Anita Sari" sheetId="41" state="visible" r:id="rId41"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Detail - Harum Nuraulia Sri Kam" sheetId="42" state="visible" r:id="rId42"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Detail - Azzahra Qyasimah" sheetId="43" state="visible" r:id="rId43"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Detail - Aupa Aznia" sheetId="44" state="visible" r:id="rId44"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Detail - Alya Nuraeni" sheetId="45" state="visible" r:id="rId45"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Detail - Siti Jenab" sheetId="46" state="visible" r:id="rId46"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Detail - Wildan" sheetId="47" state="visible" r:id="rId47"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Detail - Debi Lestari" sheetId="48" state="visible" r:id="rId48"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Detail - Hasni Sapa Al Maira" sheetId="49" state="visible" r:id="rId49"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Detail - Ilfa Alifiana Khoeruni" sheetId="50" state="visible" r:id="rId50"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Detail - Dira Rahmawati" sheetId="51" state="visible" r:id="rId51"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Detail - Nazma Kayva Gasani" sheetId="52" state="visible" r:id="rId52"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Detail - Riana Sanjaya" sheetId="53" state="visible" r:id="rId53"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Detail - Nazwa Nur Aisyah" sheetId="54" state="visible" r:id="rId54"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Detail - Ai Cinta Lestari" sheetId="55" state="visible" r:id="rId55"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Detail - Tira Fadila" sheetId="56" state="visible" r:id="rId56"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Detail - Ai Nurawaliah Al Zahra" sheetId="57" state="visible" r:id="rId57"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Detail - Ai Imas" sheetId="58" state="visible" r:id="rId58"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Detail - Syifa Haira" sheetId="59" state="visible" r:id="rId59"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Detail - Rismayanti" sheetId="60" state="visible" r:id="rId60"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Detail - Moh Pikri" sheetId="61" state="visible" r:id="rId61"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Detail - Sumiyati" sheetId="62" state="visible" r:id="rId62"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Detail - Ajeng Dwi Raissa Fitri" sheetId="63" state="visible" r:id="rId63"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Detail - Sri Ayu Wahyuni" sheetId="64" state="visible" r:id="rId64"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Detail - Risma Saparani" sheetId="65" state="visible" r:id="rId65"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Detail - Zahratul Ayesa Aulia" sheetId="66" state="visible" r:id="rId66"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Detail - Gadna Widiatni" sheetId="67" state="visible" r:id="rId67"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Detail - Devina Nayyra Fitriani" sheetId="68" state="visible" r:id="rId68"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Detail - Sulistiawati" sheetId="69" state="visible" r:id="rId69"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Detail - Sechan Khalifatunnisa" sheetId="70" state="visible" r:id="rId70"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Detail - Fitriyani" sheetId="71" state="visible" r:id="rId71"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Detail - Syabina Ayat El Akhros" sheetId="72" state="visible" r:id="rId72"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Detail - Siti Rahma Silpiana" sheetId="73" state="visible" r:id="rId73"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Detail - Teni Damayanti" sheetId="74" state="visible" r:id="rId74"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Detail - Siti Khoiriyah" sheetId="75" state="visible" r:id="rId75"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Detail - Aqila Nazil Falaq" sheetId="76" state="visible" r:id="rId76"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Detail - Resti Nurul Fadila" sheetId="77" state="visible" r:id="rId77"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Detail - Neng Oktavia Putri Agu" sheetId="78" state="visible" r:id="rId78"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Detail - Fahmi Ahmad Ramdan Alf" sheetId="79" state="visible" r:id="rId79"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Detail - Nadira Mega Rizkia" sheetId="80" state="visible" r:id="rId80"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Detail - Rita Pebriyani" sheetId="81" state="visible" r:id="rId81"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Detail - Ai Siti Muslimah" sheetId="82" state="visible" r:id="rId82"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Detail - Nani Yuliyani" sheetId="83" state="visible" r:id="rId83"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Detail - Amira Nur Aulia" sheetId="84" state="visible" r:id="rId84"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Detail - Raira Putri" sheetId="85" state="visible" r:id="rId85"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Detail - Kaila Aropatilah" sheetId="86" state="visible" r:id="rId86"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Detail - Nuri Meitri Aeni" sheetId="87" state="visible" r:id="rId87"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Detail - Nazwa Kurnia" sheetId="88" state="visible" r:id="rId88"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3. REKAP KETIDAKLENGKAPAN" sheetId="89" state="visible" r:id="rId89"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="4. CEK MANUAL GURU" sheetId="90" state="visible" r:id="rId90"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="5. DATA REKAPAN" sheetId="91" state="visible" r:id="rId91"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="7. NILAI TAMBAHAN RESOLUSI" sheetId="92" state="visible" r:id="rId92"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="6. METODE &amp; RUBRIK" sheetId="93" state="visible" r:id="rId93"/>
+    <sheet name="1. REKAP NILAI" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="2. NILAI KOMPONEN" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Detail - Wahdan Sapari" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Detail - Ahmad Fauzi" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Detail - Qiandra Kaizar Nahari" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Detail - Ilma Latifah" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Detail - Sopa Anidatul Aisah" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Detail - Jajang M Husni Mubarok" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Detail - Silvi Budia Putri" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Detail - Nurjihan" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="Detail - Dede Aprilia Kartika" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="Detail - Putri Intan Nuraeni" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="Detail - Intan Widiyanti" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="Detail - Safinah Syara Garini" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet name="Detail - Quinsya Rahmanesa Sole" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet name="Detail - Jihan Shafira Kean Put" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet name="Detail - Dhea Eka Khoerunnisa" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet name="Detail - Wulan Sundari" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet name="Detail - Wilda Azkia" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet name="Detail - Muhamad Diaz Pirdaus" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet name="Detail - Rizky Muhammad Regal S" sheetId="21" state="visible" r:id="rId21"/>
+    <sheet name="Detail - Khanza Nuraeni" sheetId="22" state="visible" r:id="rId22"/>
+    <sheet name="Detail - Ceisha Sinthia" sheetId="23" state="visible" r:id="rId23"/>
+    <sheet name="Detail - Selvi Sifa Urizqi" sheetId="24" state="visible" r:id="rId24"/>
+    <sheet name="Detail - Azmi Anugrah" sheetId="25" state="visible" r:id="rId25"/>
+    <sheet name="Detail - Indri Fitriyani" sheetId="26" state="visible" r:id="rId26"/>
+    <sheet name="Detail - Meisya Fakhriyah" sheetId="27" state="visible" r:id="rId27"/>
+    <sheet name="Detail - M Reza Huafah" sheetId="28" state="visible" r:id="rId28"/>
+    <sheet name="Detail - Syiva Widiyana Agustin" sheetId="29" state="visible" r:id="rId29"/>
+    <sheet name="Detail - Meylan Meliyanti Anast" sheetId="30" state="visible" r:id="rId30"/>
+    <sheet name="Detail - Putri Utami" sheetId="31" state="visible" r:id="rId31"/>
+    <sheet name="Detail - Kamila Apriliani" sheetId="32" state="visible" r:id="rId32"/>
+    <sheet name="Detail - Yayu Astia" sheetId="33" state="visible" r:id="rId33"/>
+    <sheet name="Detail - Wina Afriliani" sheetId="34" state="visible" r:id="rId34"/>
+    <sheet name="Detail - Jajang Nurjaman" sheetId="35" state="visible" r:id="rId35"/>
+    <sheet name="Detail - Shandika Revi Shafarud" sheetId="36" state="visible" r:id="rId36"/>
+    <sheet name="Detail - Ai Tito" sheetId="37" state="visible" r:id="rId37"/>
+    <sheet name="Detail - Merlin Aznika" sheetId="38" state="visible" r:id="rId38"/>
+    <sheet name="Detail - Neng Sri Rahayu" sheetId="39" state="visible" r:id="rId39"/>
+    <sheet name="Detail - Sindia Saputri" sheetId="40" state="visible" r:id="rId40"/>
+    <sheet name="Detail - Mutia Anita Sari" sheetId="41" state="visible" r:id="rId41"/>
+    <sheet name="Detail - Harum Nuraulia Sri Kam" sheetId="42" state="visible" r:id="rId42"/>
+    <sheet name="Detail - Azzahra Qyasimah" sheetId="43" state="visible" r:id="rId43"/>
+    <sheet name="Detail - Aupa Aznia" sheetId="44" state="visible" r:id="rId44"/>
+    <sheet name="Detail - Alya Nuraeni" sheetId="45" state="visible" r:id="rId45"/>
+    <sheet name="Detail - Siti Jenab" sheetId="46" state="visible" r:id="rId46"/>
+    <sheet name="Detail - Wildan" sheetId="47" state="visible" r:id="rId47"/>
+    <sheet name="Detail - Debi Lestari" sheetId="48" state="visible" r:id="rId48"/>
+    <sheet name="Detail - Hasni Sapa Al Maira" sheetId="49" state="visible" r:id="rId49"/>
+    <sheet name="Detail - Ilfa Alifiana Khoeruni" sheetId="50" state="visible" r:id="rId50"/>
+    <sheet name="Detail - Dira Rahmawati" sheetId="51" state="visible" r:id="rId51"/>
+    <sheet name="Detail - Nazma Kayva Gasani" sheetId="52" state="visible" r:id="rId52"/>
+    <sheet name="Detail - Riana Sanjaya" sheetId="53" state="visible" r:id="rId53"/>
+    <sheet name="Detail - Nazwa Nur Aisyah" sheetId="54" state="visible" r:id="rId54"/>
+    <sheet name="Detail - Ai Cinta Lestari" sheetId="55" state="visible" r:id="rId55"/>
+    <sheet name="Detail - Tira Fadila" sheetId="56" state="visible" r:id="rId56"/>
+    <sheet name="Detail - Ai Nurawaliah Al Zahra" sheetId="57" state="visible" r:id="rId57"/>
+    <sheet name="Detail - Ai Imas" sheetId="58" state="visible" r:id="rId58"/>
+    <sheet name="Detail - Syifa Haira" sheetId="59" state="visible" r:id="rId59"/>
+    <sheet name="Detail - Rismayanti" sheetId="60" state="visible" r:id="rId60"/>
+    <sheet name="Detail - Moh Pikri" sheetId="61" state="visible" r:id="rId61"/>
+    <sheet name="Detail - Sumiyati" sheetId="62" state="visible" r:id="rId62"/>
+    <sheet name="Detail - Ajeng Dwi Raissa Fitri" sheetId="63" state="visible" r:id="rId63"/>
+    <sheet name="Detail - Sri Ayu Wahyuni" sheetId="64" state="visible" r:id="rId64"/>
+    <sheet name="Detail - Risma Saparani" sheetId="65" state="visible" r:id="rId65"/>
+    <sheet name="Detail - Zahratul Ayesa Aulia" sheetId="66" state="visible" r:id="rId66"/>
+    <sheet name="Detail - Gadna Widiatni" sheetId="67" state="visible" r:id="rId67"/>
+    <sheet name="Detail - Devina Nayyra Fitriani" sheetId="68" state="visible" r:id="rId68"/>
+    <sheet name="Detail - Sulistiawati" sheetId="69" state="visible" r:id="rId69"/>
+    <sheet name="Detail - Sechan Khalifatunnisa" sheetId="70" state="visible" r:id="rId70"/>
+    <sheet name="Detail - Fitriyani" sheetId="71" state="visible" r:id="rId71"/>
+    <sheet name="Detail - Syabina Ayat El Akhros" sheetId="72" state="visible" r:id="rId72"/>
+    <sheet name="Detail - Siti Rahma Silpiana" sheetId="73" state="visible" r:id="rId73"/>
+    <sheet name="Detail - Teni Damayanti" sheetId="74" state="visible" r:id="rId74"/>
+    <sheet name="Detail - Siti Khoiriyah" sheetId="75" state="visible" r:id="rId75"/>
+    <sheet name="Detail - Aqila Nazil Falaq" sheetId="76" state="visible" r:id="rId76"/>
+    <sheet name="Detail - Resti Nurul Fadila" sheetId="77" state="visible" r:id="rId77"/>
+    <sheet name="Detail - Neng Oktavia Putri Agu" sheetId="78" state="visible" r:id="rId78"/>
+    <sheet name="Detail - Fahmi Ahmad Ramdan Alf" sheetId="79" state="visible" r:id="rId79"/>
+    <sheet name="Detail - Nadira Mega Rizkia" sheetId="80" state="visible" r:id="rId80"/>
+    <sheet name="Detail - Rita Pebriyani" sheetId="81" state="visible" r:id="rId81"/>
+    <sheet name="Detail - Ai Siti Muslimah" sheetId="82" state="visible" r:id="rId82"/>
+    <sheet name="Detail - Nani Yuliyani" sheetId="83" state="visible" r:id="rId83"/>
+    <sheet name="Detail - Amira Nur Aulia" sheetId="84" state="visible" r:id="rId84"/>
+    <sheet name="Detail - Raira Putri" sheetId="85" state="visible" r:id="rId85"/>
+    <sheet name="Detail - Kaila Aropatilah" sheetId="86" state="visible" r:id="rId86"/>
+    <sheet name="Detail - Nuri Meitri Aeni" sheetId="87" state="visible" r:id="rId87"/>
+    <sheet name="Detail - Nazwa Kurnia" sheetId="88" state="visible" r:id="rId88"/>
+    <sheet name="3. REKAP KETIDAKLENGKAPAN" sheetId="89" state="visible" r:id="rId89"/>
+    <sheet name="4. CEK MANUAL GURU" sheetId="90" state="visible" r:id="rId90"/>
+    <sheet name="5. DATA REKAPAN" sheetId="91" state="visible" r:id="rId91"/>
+    <sheet name="7. NILAI TAMBAHAN RESOLUSI" sheetId="92" state="visible" r:id="rId92"/>
+    <sheet name="6. METODE &amp; RUBRIK" sheetId="93" state="visible" r:id="rId93"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>

</xml_diff>